<commit_message>
fix(research): clarify zero-score ranking placeholders
</commit_message>
<xml_diff>
--- a/research/phase-4/deliveries/2026-07-16_phase-4-v6-final/Phase_4_Country_Product_Demand_Ranking_v6.xlsx
+++ b/research/phase-4/deliveries/2026-07-16_phase-4-v6-final/Phase_4_Country_Product_Demand_Ranking_v6.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engine Top 3" sheetId="1" r:id="R4da3ff4f0f1443e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aftermarket Offer" sheetId="2" r:id="R0489a5143b9e45cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engine Top 3" sheetId="1" r:id="R5b8ed684a1514136"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aftermarket Offer" sheetId="2" r:id="R48ad8fbecf854e6b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -497,7 +497,7 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="J6" s="7" t="str">
-        <x:v>Frozen Phase 4 direction</x:v>
+        <x:v>Zero-score placeholder; no evidence-supported direction</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Low</x:v>
       </x:c>
       <x:c r="J7" s="7" t="str">
-        <x:v>Frozen Phase 4 direction</x:v>
+        <x:v>Zero-score placeholder; no evidence-supported direction</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">

</xml_diff>